<commit_message>
Preserve long archive identities and publish updated data
</commit_message>
<xml_diff>
--- a/benchmark_data/10Y国债地债YTM.xlsx
+++ b/benchmark_data/10Y国债地债YTM.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1625"/>
+  <dimension ref="A1:C1631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18313,6 +18313,70 @@
         <v>1.77</v>
       </c>
     </row>
+    <row r="1626">
+      <c r="A1626" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1626" t="n">
+        <v>1.6888</v>
+      </c>
+      <c r="C1626" t="n">
+        <v>1.765</v>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1627" t="n">
+        <v>1.6865</v>
+      </c>
+      <c r="C1627" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1628" t="n">
+        <v>1.6858</v>
+      </c>
+      <c r="C1628" t="n">
+        <v>1.7569</v>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1629" t="n">
+        <v>1.6862</v>
+      </c>
+      <c r="C1629" t="n">
+        <v>1.7569</v>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1630" t="n">
+        <v>1.682</v>
+      </c>
+      <c r="C1630" t="n">
+        <v>1.755</v>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1631" t="n">
+        <v>1.6818</v>
+      </c>
+      <c r="C1631" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>